<commit_message>
Move T15 finals to separate worksheet
</commit_message>
<xml_diff>
--- a/nbv_turniermodi_excel/T15_8 Spieler zwei Vierergruppen Kalender-Vorlage.xlsx
+++ b/nbv_turniermodi_excel/T15_8 Spieler zwei Vierergruppen Kalender-Vorlage.xlsx
@@ -9,11 +9,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnehmer" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV Export" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finalrunde" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau'!$A$1:$J$81</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau'!$A$1:$P$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Teilnehmer'!$A$1:$F$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'CSV Export'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Finalrunde'!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -25,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -83,8 +85,13 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -131,8 +138,13 @@
         <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -493,12 +505,148 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="center"/>
@@ -674,6 +822,29 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1013,7 +1184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P84"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="18" customWidth="1" style="19" min="1" max="1"/>
@@ -2164,1471 +2335,145 @@
     <row r="34" ht="22" customHeight="1" s="19"/>
     <row r="35" ht="22" customHeight="1" s="19"/>
     <row r="36" ht="22" customHeight="1" s="19"/>
-    <row r="37" ht="24" customHeight="1" s="19">
-      <c r="A37" s="55" t="inlineStr">
-        <is>
-          <t>Finalrunde - Halbfinale</t>
-        </is>
-      </c>
-      <c r="K37" s="56" t="n"/>
-      <c r="L37" s="56" t="n"/>
-      <c r="M37" s="56" t="n"/>
-      <c r="N37" s="56" t="n"/>
-      <c r="O37" s="56" t="n"/>
-      <c r="P37" s="56" t="n"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" s="19">
-      <c r="A38" s="57" t="inlineStr">
-        <is>
-          <t>Spieler</t>
-        </is>
-      </c>
-      <c r="B38" s="57" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="C38" s="57" t="inlineStr">
-        <is>
-          <t>1. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="D38" s="58" t="n"/>
-      <c r="E38" s="57" t="inlineStr">
-        <is>
-          <t>2. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="F38" s="58" t="n"/>
-      <c r="G38" s="57" t="inlineStr">
-        <is>
-          <t>1. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="H38" s="58" t="n"/>
-      <c r="I38" s="57" t="inlineStr">
-        <is>
-          <t>2. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="J38" s="58" t="n"/>
-      <c r="K38" s="56" t="n"/>
-      <c r="L38" s="56" t="n"/>
-      <c r="M38" s="56" t="n"/>
-      <c r="N38" s="56" t="n"/>
-      <c r="O38" s="56" t="n"/>
-      <c r="P38" s="56" t="n"/>
-    </row>
-    <row r="39" ht="22" customHeight="1" s="19">
-      <c r="A39" s="59" t="inlineStr">
-        <is>
-          <t>1. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="B39" s="59" t="inlineStr"/>
-      <c r="C39" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="D39" s="61" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="E39" s="62" t="n"/>
-      <c r="F39" s="62" t="n"/>
-      <c r="G39" s="63" t="n"/>
-      <c r="H39" s="63" t="n"/>
-      <c r="I39" s="63" t="n"/>
-      <c r="J39" s="63" t="n"/>
-      <c r="K39" s="64" t="n"/>
-      <c r="L39" s="64" t="n"/>
-      <c r="M39" s="64" t="n"/>
-      <c r="N39" s="56" t="n"/>
-      <c r="O39" s="56" t="n"/>
-      <c r="P39" s="56" t="n"/>
-    </row>
-    <row r="40" ht="22" customHeight="1" s="19">
-      <c r="A40" s="59" t="n"/>
-      <c r="B40" s="59" t="n"/>
-      <c r="C40" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="D40" s="60" t="n"/>
-      <c r="E40" s="62">
-        <f>IF(OR(E39="",C42=""),"",IF(E39&gt;C42,2,IF(E39&lt;C42,0,1)))</f>
-        <v/>
-      </c>
-      <c r="F40" s="62" t="n"/>
-      <c r="G40" s="63" t="n"/>
-      <c r="H40" s="63" t="n"/>
-      <c r="I40" s="63" t="n"/>
-      <c r="J40" s="63" t="n"/>
-      <c r="K40" s="64" t="n"/>
-      <c r="L40" s="64" t="n"/>
-      <c r="M40" s="64" t="n"/>
-      <c r="N40" s="56" t="n"/>
-      <c r="O40" s="56" t="n"/>
-      <c r="P40" s="56" t="n"/>
-    </row>
-    <row r="41" ht="22" customHeight="1" s="19">
-      <c r="A41" s="59" t="n"/>
-      <c r="B41" s="59" t="n"/>
-      <c r="C41" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="D41" s="61" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="E41" s="62">
-        <f>IF(F39&gt;0,TRUNC(E39/F39,3),"")</f>
-        <v/>
-      </c>
-      <c r="F41" s="62" t="n"/>
-      <c r="G41" s="63" t="n"/>
-      <c r="H41" s="63" t="n"/>
-      <c r="I41" s="63" t="n"/>
-      <c r="J41" s="63" t="n"/>
-      <c r="K41" s="64" t="n"/>
-      <c r="L41" s="64" t="n"/>
-      <c r="M41" s="64" t="n"/>
-      <c r="N41" s="56" t="n"/>
-      <c r="O41" s="56" t="n"/>
-      <c r="P41" s="56" t="n"/>
-    </row>
-    <row r="42" ht="22" customHeight="1" s="19">
-      <c r="A42" s="59" t="inlineStr">
-        <is>
-          <t>2. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="B42" s="59" t="inlineStr"/>
-      <c r="C42" s="65" t="n"/>
-      <c r="D42" s="62" t="n"/>
-      <c r="E42" s="61" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="F42" s="61" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="G42" s="63" t="n"/>
-      <c r="H42" s="63" t="n"/>
-      <c r="I42" s="63" t="n"/>
-      <c r="J42" s="63" t="n"/>
-      <c r="K42" s="64" t="n"/>
-      <c r="L42" s="64" t="n"/>
-      <c r="M42" s="64" t="n"/>
-      <c r="N42" s="56" t="n"/>
-      <c r="O42" s="56" t="n"/>
-      <c r="P42" s="56" t="n"/>
-    </row>
-    <row r="43" ht="22" customHeight="1" s="19">
-      <c r="A43" s="59" t="n"/>
-      <c r="B43" s="59" t="n"/>
-      <c r="C43" s="65">
-        <f>IF(OR(C42="",E39=""),"",IF(C42&gt;E39,2,IF(C42&lt;E39,0,1)))</f>
-        <v/>
-      </c>
-      <c r="D43" s="65" t="n"/>
-      <c r="E43" s="61" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="F43" s="61" t="n"/>
-      <c r="G43" s="63" t="n"/>
-      <c r="H43" s="63" t="n"/>
-      <c r="I43" s="63" t="n"/>
-      <c r="J43" s="63" t="n"/>
-      <c r="K43" s="64" t="n"/>
-      <c r="L43" s="64" t="n"/>
-      <c r="M43" s="64" t="n"/>
-      <c r="N43" s="56" t="n"/>
-      <c r="O43" s="56" t="n"/>
-      <c r="P43" s="56" t="n"/>
-    </row>
-    <row r="44" ht="22" customHeight="1" s="19">
-      <c r="A44" s="59" t="n"/>
-      <c r="B44" s="59" t="n"/>
-      <c r="C44" s="65">
-        <f>IF(D42&gt;0,TRUNC(C42/D42,3),"")</f>
-        <v/>
-      </c>
-      <c r="D44" s="62" t="n"/>
-      <c r="E44" s="61" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="F44" s="61" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="G44" s="63" t="n"/>
-      <c r="H44" s="63" t="n"/>
-      <c r="I44" s="63" t="n"/>
-      <c r="J44" s="63" t="n"/>
-      <c r="K44" s="64" t="n"/>
-      <c r="L44" s="64" t="n"/>
-      <c r="M44" s="64" t="n"/>
-      <c r="N44" s="56" t="n"/>
-      <c r="O44" s="56" t="n"/>
-      <c r="P44" s="56" t="n"/>
-    </row>
-    <row r="45" ht="22" customHeight="1" s="19">
-      <c r="A45" s="59" t="inlineStr">
-        <is>
-          <t>1. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="B45" s="59" t="inlineStr"/>
-      <c r="C45" s="66" t="n"/>
-      <c r="D45" s="66" t="n"/>
-      <c r="E45" s="66" t="n"/>
-      <c r="F45" s="66" t="n"/>
-      <c r="G45" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="H45" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="I45" s="65" t="n"/>
-      <c r="J45" s="65" t="n"/>
-      <c r="K45" s="56" t="n"/>
-      <c r="L45" s="56" t="n"/>
-      <c r="M45" s="56" t="n"/>
-      <c r="N45" s="56" t="n"/>
-      <c r="O45" s="56" t="n"/>
-      <c r="P45" s="56" t="n"/>
-    </row>
-    <row r="46" ht="22" customHeight="1" s="19">
-      <c r="A46" s="59" t="n"/>
-      <c r="B46" s="59" t="n"/>
-      <c r="C46" s="66" t="n"/>
-      <c r="D46" s="66" t="n"/>
-      <c r="E46" s="66" t="n"/>
-      <c r="F46" s="66" t="n"/>
-      <c r="G46" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="H46" s="60" t="n"/>
-      <c r="I46" s="65">
-        <f>IF(OR(I45="",G48=""),"",IF(I45&gt;G48,2,IF(I45&lt;G48,0,1)))</f>
-        <v/>
-      </c>
-      <c r="J46" s="65" t="n"/>
-      <c r="K46" s="56" t="n"/>
-      <c r="L46" s="56" t="n"/>
-      <c r="M46" s="56" t="n"/>
-      <c r="N46" s="56" t="n"/>
-      <c r="O46" s="56" t="n"/>
-      <c r="P46" s="56" t="n"/>
-    </row>
-    <row r="47" ht="22" customHeight="1" s="19">
-      <c r="A47" s="59" t="n"/>
-      <c r="B47" s="59" t="n"/>
-      <c r="C47" s="66" t="n"/>
-      <c r="D47" s="66" t="n"/>
-      <c r="E47" s="66" t="n"/>
-      <c r="F47" s="66" t="n"/>
-      <c r="G47" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="H47" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="I47" s="65">
-        <f>IF(J45&gt;0,TRUNC(I45/J45,3),"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="65" t="n"/>
-      <c r="K47" s="56" t="n"/>
-      <c r="L47" s="56" t="n"/>
-      <c r="M47" s="56" t="n"/>
-      <c r="N47" s="56" t="n"/>
-      <c r="O47" s="56" t="n"/>
-      <c r="P47" s="56" t="n"/>
-    </row>
-    <row r="48" ht="22" customHeight="1" s="19">
-      <c r="A48" s="59" t="inlineStr">
-        <is>
-          <t>2. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="B48" s="59" t="inlineStr"/>
-      <c r="C48" s="66" t="n"/>
-      <c r="D48" s="66" t="n"/>
-      <c r="E48" s="66" t="n"/>
-      <c r="F48" s="66" t="n"/>
-      <c r="G48" s="65" t="n"/>
-      <c r="H48" s="65" t="n"/>
-      <c r="I48" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="J48" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="K48" s="56" t="n"/>
-      <c r="L48" s="56" t="n"/>
-      <c r="M48" s="56" t="n"/>
-      <c r="N48" s="56" t="n"/>
-      <c r="O48" s="56" t="n"/>
-      <c r="P48" s="56" t="n"/>
-    </row>
-    <row r="49" ht="22" customHeight="1" s="19">
-      <c r="A49" s="59" t="n"/>
-      <c r="B49" s="59" t="n"/>
-      <c r="C49" s="66" t="n"/>
-      <c r="D49" s="66" t="n"/>
-      <c r="E49" s="66" t="n"/>
-      <c r="F49" s="66" t="n"/>
-      <c r="G49" s="65">
-        <f>IF(OR(G48="",I45=""),"",IF(G48&gt;I45,2,IF(G48&lt;I45,0,1)))</f>
-        <v/>
-      </c>
-      <c r="H49" s="65" t="n"/>
-      <c r="I49" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="J49" s="60" t="n"/>
-      <c r="K49" s="56" t="n"/>
-      <c r="L49" s="56" t="n"/>
-      <c r="M49" s="56" t="n"/>
-      <c r="N49" s="56" t="n"/>
-      <c r="O49" s="56" t="n"/>
-      <c r="P49" s="56" t="n"/>
-    </row>
-    <row r="50" ht="22" customHeight="1" s="19">
-      <c r="A50" s="59" t="n"/>
-      <c r="B50" s="59" t="n"/>
-      <c r="C50" s="66" t="n"/>
-      <c r="D50" s="66" t="n"/>
-      <c r="E50" s="66" t="n"/>
-      <c r="F50" s="66" t="n"/>
-      <c r="G50" s="65">
-        <f>IF(H48&gt;0,TRUNC(G48/H48,3),"")</f>
-        <v/>
-      </c>
-      <c r="H50" s="65" t="n"/>
-      <c r="I50" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="J50" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="K50" s="56" t="n"/>
-      <c r="L50" s="56" t="n"/>
-      <c r="M50" s="56" t="n"/>
-      <c r="N50" s="56" t="n"/>
-      <c r="O50" s="56" t="n"/>
-      <c r="P50" s="56" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="56" t="n"/>
-      <c r="B51" s="56" t="n"/>
-      <c r="C51" s="56" t="n"/>
-      <c r="D51" s="56" t="n"/>
-      <c r="E51" s="56" t="n"/>
-      <c r="F51" s="56" t="n"/>
-      <c r="G51" s="56" t="n"/>
-      <c r="H51" s="56" t="n"/>
-      <c r="I51" s="56" t="n"/>
-      <c r="J51" s="56" t="n"/>
-      <c r="K51" s="56" t="n"/>
-      <c r="L51" s="56" t="n"/>
-      <c r="M51" s="56" t="n"/>
-      <c r="N51" s="56" t="n"/>
-      <c r="O51" s="56" t="n"/>
-      <c r="P51" s="56" t="n"/>
-    </row>
-    <row r="52" ht="24" customHeight="1" s="19">
-      <c r="A52" s="55" t="inlineStr">
-        <is>
-          <t>Finalrunde - Platzierung 5-8</t>
-        </is>
-      </c>
-      <c r="K52" s="56" t="n"/>
-      <c r="L52" s="56" t="n"/>
-      <c r="M52" s="56" t="n"/>
-      <c r="N52" s="56" t="n"/>
-      <c r="O52" s="56" t="n"/>
-      <c r="P52" s="56" t="n"/>
-    </row>
-    <row r="53" ht="24" customHeight="1" s="19">
-      <c r="A53" s="57" t="inlineStr">
-        <is>
-          <t>Spieler</t>
-        </is>
-      </c>
-      <c r="B53" s="57" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="C53" s="57" t="inlineStr">
-        <is>
-          <t>3. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="D53" s="58" t="n"/>
-      <c r="E53" s="57" t="inlineStr">
-        <is>
-          <t>3. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="F53" s="58" t="n"/>
-      <c r="G53" s="57" t="inlineStr">
-        <is>
-          <t>4. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="H53" s="58" t="n"/>
-      <c r="I53" s="57" t="inlineStr">
-        <is>
-          <t>4. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="J53" s="58" t="n"/>
-      <c r="K53" s="56" t="n"/>
-      <c r="L53" s="56" t="n"/>
-      <c r="M53" s="56" t="n"/>
-      <c r="N53" s="56" t="n"/>
-      <c r="O53" s="56" t="n"/>
-      <c r="P53" s="56" t="n"/>
-    </row>
-    <row r="54" ht="22" customHeight="1" s="19">
-      <c r="A54" s="59" t="inlineStr">
-        <is>
-          <t>3. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="B54" s="59" t="inlineStr"/>
-      <c r="C54" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="D54" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="E54" s="65" t="n"/>
-      <c r="F54" s="65" t="n"/>
-      <c r="G54" s="66" t="n"/>
-      <c r="H54" s="66" t="n"/>
-      <c r="I54" s="66" t="n"/>
-      <c r="J54" s="66" t="n"/>
-      <c r="K54" s="56" t="n"/>
-      <c r="L54" s="56" t="n"/>
-      <c r="M54" s="56" t="n"/>
-      <c r="N54" s="56" t="n"/>
-      <c r="O54" s="56" t="n"/>
-      <c r="P54" s="56" t="n"/>
-    </row>
-    <row r="55" ht="22" customHeight="1" s="19">
-      <c r="A55" s="59" t="n"/>
-      <c r="B55" s="59" t="n"/>
-      <c r="C55" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="D55" s="60" t="n"/>
-      <c r="E55" s="65">
-        <f>IF(OR(E54="",C57=""),"",IF(E54&gt;C57,2,IF(E54&lt;C57,0,1)))</f>
-        <v/>
-      </c>
-      <c r="F55" s="65" t="n"/>
-      <c r="G55" s="66" t="n"/>
-      <c r="H55" s="66" t="n"/>
-      <c r="I55" s="66" t="n"/>
-      <c r="J55" s="66" t="n"/>
-      <c r="K55" s="56" t="n"/>
-      <c r="L55" s="56" t="n"/>
-      <c r="M55" s="56" t="n"/>
-      <c r="N55" s="56" t="n"/>
-      <c r="O55" s="56" t="n"/>
-      <c r="P55" s="56" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1" s="19">
-      <c r="A56" s="59" t="n"/>
-      <c r="B56" s="59" t="n"/>
-      <c r="C56" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="D56" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="E56" s="65">
-        <f>IF(F54&gt;0,TRUNC(E54/F54,3),"")</f>
-        <v/>
-      </c>
-      <c r="F56" s="65" t="n"/>
-      <c r="G56" s="66" t="n"/>
-      <c r="H56" s="66" t="n"/>
-      <c r="I56" s="66" t="n"/>
-      <c r="J56" s="66" t="n"/>
-      <c r="K56" s="56" t="n"/>
-      <c r="L56" s="56" t="n"/>
-      <c r="M56" s="56" t="n"/>
-      <c r="N56" s="56" t="n"/>
-      <c r="O56" s="56" t="n"/>
-      <c r="P56" s="56" t="n"/>
-    </row>
-    <row r="57" ht="22" customHeight="1" s="19">
-      <c r="A57" s="59" t="inlineStr">
-        <is>
-          <t>3. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="B57" s="59" t="inlineStr"/>
-      <c r="C57" s="65" t="n"/>
-      <c r="D57" s="65" t="n"/>
-      <c r="E57" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="F57" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="G57" s="66" t="n"/>
-      <c r="H57" s="66" t="n"/>
-      <c r="I57" s="66" t="n"/>
-      <c r="J57" s="66" t="n"/>
-      <c r="K57" s="56" t="n"/>
-      <c r="L57" s="56" t="n"/>
-      <c r="M57" s="56" t="n"/>
-      <c r="N57" s="56" t="n"/>
-      <c r="O57" s="56" t="n"/>
-      <c r="P57" s="56" t="n"/>
-    </row>
-    <row r="58" ht="22" customHeight="1" s="19">
-      <c r="A58" s="59" t="n"/>
-      <c r="B58" s="59" t="n"/>
-      <c r="C58" s="65">
-        <f>IF(OR(C57="",E54=""),"",IF(C57&gt;E54,2,IF(C57&lt;E54,0,1)))</f>
-        <v/>
-      </c>
-      <c r="D58" s="65" t="n"/>
-      <c r="E58" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="F58" s="60" t="n"/>
-      <c r="G58" s="66" t="n"/>
-      <c r="H58" s="66" t="n"/>
-      <c r="I58" s="66" t="n"/>
-      <c r="J58" s="66" t="n"/>
-      <c r="K58" s="56" t="n"/>
-      <c r="L58" s="56" t="n"/>
-      <c r="M58" s="56" t="n"/>
-      <c r="N58" s="56" t="n"/>
-      <c r="O58" s="56" t="n"/>
-      <c r="P58" s="56" t="n"/>
-    </row>
-    <row r="59" ht="22" customHeight="1" s="19">
-      <c r="A59" s="59" t="n"/>
-      <c r="B59" s="59" t="n"/>
-      <c r="C59" s="65">
-        <f>IF(D57&gt;0,TRUNC(C57/D57,3),"")</f>
-        <v/>
-      </c>
-      <c r="D59" s="65" t="n"/>
-      <c r="E59" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="F59" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="G59" s="66" t="n"/>
-      <c r="H59" s="66" t="n"/>
-      <c r="I59" s="66" t="n"/>
-      <c r="J59" s="66" t="n"/>
-      <c r="K59" s="56" t="n"/>
-      <c r="L59" s="56" t="n"/>
-      <c r="M59" s="56" t="n"/>
-      <c r="N59" s="56" t="n"/>
-      <c r="O59" s="56" t="n"/>
-      <c r="P59" s="56" t="n"/>
-    </row>
-    <row r="60" ht="22" customHeight="1" s="19">
-      <c r="A60" s="59" t="inlineStr">
-        <is>
-          <t>4. Gruppe 1</t>
-        </is>
-      </c>
-      <c r="B60" s="59" t="inlineStr"/>
-      <c r="C60" s="66" t="n"/>
-      <c r="D60" s="66" t="n"/>
-      <c r="E60" s="66" t="n"/>
-      <c r="F60" s="66" t="n"/>
-      <c r="G60" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="H60" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="I60" s="65" t="n"/>
-      <c r="J60" s="65" t="n"/>
-      <c r="K60" s="56" t="n"/>
-      <c r="L60" s="56" t="n"/>
-      <c r="M60" s="56" t="n"/>
-      <c r="N60" s="56" t="n"/>
-      <c r="O60" s="56" t="n"/>
-      <c r="P60" s="56" t="n"/>
-    </row>
-    <row r="61" ht="22" customHeight="1" s="19">
-      <c r="A61" s="59" t="n"/>
-      <c r="B61" s="59" t="n"/>
-      <c r="C61" s="66" t="n"/>
-      <c r="D61" s="66" t="n"/>
-      <c r="E61" s="66" t="n"/>
-      <c r="F61" s="66" t="n"/>
-      <c r="G61" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="H61" s="60" t="n"/>
-      <c r="I61" s="65">
-        <f>IF(OR(I60="",G63=""),"",IF(I60&gt;G63,2,IF(I60&lt;G63,0,1)))</f>
-        <v/>
-      </c>
-      <c r="J61" s="65" t="n"/>
-      <c r="K61" s="56" t="n"/>
-      <c r="L61" s="56" t="n"/>
-      <c r="M61" s="56" t="n"/>
-      <c r="N61" s="56" t="n"/>
-      <c r="O61" s="56" t="n"/>
-      <c r="P61" s="56" t="n"/>
-    </row>
-    <row r="62" ht="22" customHeight="1" s="19">
-      <c r="A62" s="59" t="n"/>
-      <c r="B62" s="59" t="n"/>
-      <c r="C62" s="66" t="n"/>
-      <c r="D62" s="66" t="n"/>
-      <c r="E62" s="66" t="n"/>
-      <c r="F62" s="66" t="n"/>
-      <c r="G62" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="H62" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="I62" s="65">
-        <f>IF(J60&gt;0,TRUNC(I60/J60,3),"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="65" t="n"/>
-      <c r="K62" s="56" t="n"/>
-      <c r="L62" s="56" t="n"/>
-      <c r="M62" s="56" t="n"/>
-      <c r="N62" s="56" t="n"/>
-      <c r="O62" s="56" t="n"/>
-      <c r="P62" s="56" t="n"/>
-    </row>
-    <row r="63" ht="22" customHeight="1" s="19">
-      <c r="A63" s="59" t="inlineStr">
-        <is>
-          <t>4. Gruppe 2</t>
-        </is>
-      </c>
-      <c r="B63" s="59" t="inlineStr"/>
-      <c r="C63" s="66" t="n"/>
-      <c r="D63" s="66" t="n"/>
-      <c r="E63" s="66" t="n"/>
-      <c r="F63" s="66" t="n"/>
-      <c r="G63" s="65" t="n"/>
-      <c r="H63" s="65" t="n"/>
-      <c r="I63" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="J63" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="K63" s="56" t="n"/>
-      <c r="L63" s="56" t="n"/>
-      <c r="M63" s="56" t="n"/>
-      <c r="N63" s="56" t="n"/>
-      <c r="O63" s="56" t="n"/>
-      <c r="P63" s="56" t="n"/>
-    </row>
-    <row r="64" ht="22" customHeight="1" s="19">
-      <c r="A64" s="59" t="n"/>
-      <c r="B64" s="59" t="n"/>
-      <c r="C64" s="66" t="n"/>
-      <c r="D64" s="66" t="n"/>
-      <c r="E64" s="66" t="n"/>
-      <c r="F64" s="66" t="n"/>
-      <c r="G64" s="65">
-        <f>IF(OR(G63="",I60=""),"",IF(G63&gt;I60,2,IF(G63&lt;I60,0,1)))</f>
-        <v/>
-      </c>
-      <c r="H64" s="65" t="n"/>
-      <c r="I64" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="J64" s="60" t="n"/>
-      <c r="K64" s="56" t="n"/>
-      <c r="L64" s="56" t="n"/>
-      <c r="M64" s="56" t="n"/>
-      <c r="N64" s="56" t="n"/>
-      <c r="O64" s="56" t="n"/>
-      <c r="P64" s="56" t="n"/>
-    </row>
-    <row r="65" ht="22" customHeight="1" s="19">
-      <c r="A65" s="59" t="n"/>
-      <c r="B65" s="59" t="n"/>
-      <c r="C65" s="66" t="n"/>
-      <c r="D65" s="66" t="n"/>
-      <c r="E65" s="66" t="n"/>
-      <c r="F65" s="66" t="n"/>
-      <c r="G65" s="65">
-        <f>IF(H63&gt;0,TRUNC(G63/H63,3),"")</f>
-        <v/>
-      </c>
-      <c r="H65" s="65" t="n"/>
-      <c r="I65" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="J65" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="K65" s="56" t="n"/>
-      <c r="L65" s="56" t="n"/>
-      <c r="M65" s="56" t="n"/>
-      <c r="N65" s="56" t="n"/>
-      <c r="O65" s="56" t="n"/>
-      <c r="P65" s="56" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="56" t="n"/>
-      <c r="B66" s="56" t="n"/>
-      <c r="C66" s="56" t="n"/>
-      <c r="D66" s="56" t="n"/>
-      <c r="E66" s="56" t="n"/>
-      <c r="F66" s="56" t="n"/>
-      <c r="G66" s="56" t="n"/>
-      <c r="H66" s="56" t="n"/>
-      <c r="I66" s="56" t="n"/>
-      <c r="J66" s="56" t="n"/>
-      <c r="K66" s="56" t="n"/>
-      <c r="L66" s="56" t="n"/>
-      <c r="M66" s="56" t="n"/>
-      <c r="N66" s="56" t="n"/>
-      <c r="O66" s="56" t="n"/>
-      <c r="P66" s="56" t="n"/>
-    </row>
-    <row r="67" ht="24" customHeight="1" s="19">
-      <c r="A67" s="55" t="inlineStr">
-        <is>
-          <t>Finalrunde - Endspiele</t>
-        </is>
-      </c>
-      <c r="K67" s="56" t="n"/>
-      <c r="L67" s="56" t="n"/>
-      <c r="M67" s="56" t="n"/>
-      <c r="N67" s="56" t="n"/>
-      <c r="O67" s="56" t="n"/>
-      <c r="P67" s="56" t="n"/>
-    </row>
-    <row r="68" ht="24" customHeight="1" s="19">
-      <c r="A68" s="57" t="inlineStr">
-        <is>
-          <t>Spieler</t>
-        </is>
-      </c>
-      <c r="B68" s="57" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="C68" s="57" t="inlineStr">
-        <is>
-          <t>Sieger HF1</t>
-        </is>
-      </c>
-      <c r="D68" s="58" t="n"/>
-      <c r="E68" s="57" t="inlineStr">
-        <is>
-          <t>Sieger HF2</t>
-        </is>
-      </c>
-      <c r="F68" s="58" t="n"/>
-      <c r="G68" s="57" t="inlineStr">
-        <is>
-          <t>Verlierer HF1</t>
-        </is>
-      </c>
-      <c r="H68" s="58" t="n"/>
-      <c r="I68" s="57" t="inlineStr">
-        <is>
-          <t>Verlierer HF2</t>
-        </is>
-      </c>
-      <c r="J68" s="58" t="n"/>
-      <c r="K68" s="56" t="n"/>
-      <c r="L68" s="56" t="n"/>
-      <c r="M68" s="56" t="n"/>
-      <c r="N68" s="56" t="n"/>
-      <c r="O68" s="56" t="n"/>
-      <c r="P68" s="56" t="n"/>
-    </row>
-    <row r="69" ht="22" customHeight="1" s="19">
-      <c r="A69" s="59" t="inlineStr">
-        <is>
-          <t>Sieger HF1</t>
-        </is>
-      </c>
-      <c r="B69" s="59" t="inlineStr"/>
-      <c r="C69" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="D69" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="E69" s="65" t="n"/>
-      <c r="F69" s="65" t="n"/>
-      <c r="G69" s="66" t="n"/>
-      <c r="H69" s="66" t="n"/>
-      <c r="I69" s="66" t="n"/>
-      <c r="J69" s="66" t="n"/>
-      <c r="K69" s="56" t="n"/>
-      <c r="L69" s="56" t="n"/>
-      <c r="M69" s="56" t="n"/>
-      <c r="N69" s="56" t="n"/>
-      <c r="O69" s="56" t="n"/>
-      <c r="P69" s="56" t="n"/>
-    </row>
-    <row r="70" ht="22" customHeight="1" s="19">
-      <c r="A70" s="59" t="n"/>
-      <c r="B70" s="59" t="n"/>
-      <c r="C70" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="D70" s="60" t="n"/>
-      <c r="E70" s="65">
-        <f>IF(OR(E69="",C72=""),"",IF(E69&gt;C72,2,IF(E69&lt;C72,0,1)))</f>
-        <v/>
-      </c>
-      <c r="F70" s="65" t="n"/>
-      <c r="G70" s="66" t="n"/>
-      <c r="H70" s="66" t="n"/>
-      <c r="I70" s="66" t="n"/>
-      <c r="J70" s="66" t="n"/>
-      <c r="K70" s="56" t="n"/>
-      <c r="L70" s="56" t="n"/>
-      <c r="M70" s="56" t="n"/>
-      <c r="N70" s="56" t="n"/>
-      <c r="O70" s="56" t="n"/>
-      <c r="P70" s="56" t="n"/>
-    </row>
-    <row r="71" ht="22" customHeight="1" s="19">
-      <c r="A71" s="59" t="n"/>
-      <c r="B71" s="59" t="n"/>
-      <c r="C71" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="D71" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="E71" s="65">
-        <f>IF(F69&gt;0,TRUNC(E69/F69,3),"")</f>
-        <v/>
-      </c>
-      <c r="F71" s="65" t="n"/>
-      <c r="G71" s="66" t="n"/>
-      <c r="H71" s="66" t="n"/>
-      <c r="I71" s="66" t="n"/>
-      <c r="J71" s="66" t="n"/>
-      <c r="K71" s="56" t="n"/>
-      <c r="L71" s="56" t="n"/>
-      <c r="M71" s="56" t="n"/>
-      <c r="N71" s="56" t="n"/>
-      <c r="O71" s="56" t="n"/>
-      <c r="P71" s="56" t="n"/>
-    </row>
-    <row r="72" ht="22" customHeight="1" s="19">
-      <c r="A72" s="59" t="inlineStr">
-        <is>
-          <t>Sieger HF2</t>
-        </is>
-      </c>
-      <c r="B72" s="59" t="inlineStr"/>
-      <c r="C72" s="65" t="n"/>
-      <c r="D72" s="65" t="n"/>
-      <c r="E72" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="F72" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="G72" s="66" t="n"/>
-      <c r="H72" s="66" t="n"/>
-      <c r="I72" s="66" t="n"/>
-      <c r="J72" s="66" t="n"/>
-      <c r="K72" s="56" t="n"/>
-      <c r="L72" s="56" t="n"/>
-      <c r="M72" s="56" t="n"/>
-      <c r="N72" s="56" t="n"/>
-      <c r="O72" s="56" t="n"/>
-      <c r="P72" s="56" t="n"/>
-    </row>
-    <row r="73" ht="22" customHeight="1" s="19">
-      <c r="A73" s="59" t="n"/>
-      <c r="B73" s="59" t="n"/>
-      <c r="C73" s="65">
-        <f>IF(OR(C72="",E69=""),"",IF(C72&gt;E69,2,IF(C72&lt;E69,0,1)))</f>
-        <v/>
-      </c>
-      <c r="D73" s="65" t="n"/>
-      <c r="E73" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="F73" s="60" t="n"/>
-      <c r="G73" s="66" t="n"/>
-      <c r="H73" s="66" t="n"/>
-      <c r="I73" s="66" t="n"/>
-      <c r="J73" s="66" t="n"/>
-      <c r="K73" s="56" t="n"/>
-      <c r="L73" s="56" t="n"/>
-      <c r="M73" s="56" t="n"/>
-      <c r="N73" s="56" t="n"/>
-      <c r="O73" s="56" t="n"/>
-      <c r="P73" s="56" t="n"/>
-    </row>
-    <row r="74" ht="22" customHeight="1" s="19">
-      <c r="A74" s="59" t="n"/>
-      <c r="B74" s="59" t="n"/>
-      <c r="C74" s="65">
-        <f>IF(D72&gt;0,TRUNC(C72/D72,3),"")</f>
-        <v/>
-      </c>
-      <c r="D74" s="65" t="n"/>
-      <c r="E74" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="F74" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="G74" s="66" t="n"/>
-      <c r="H74" s="66" t="n"/>
-      <c r="I74" s="66" t="n"/>
-      <c r="J74" s="66" t="n"/>
-      <c r="K74" s="56" t="n"/>
-      <c r="L74" s="56" t="n"/>
-      <c r="M74" s="56" t="n"/>
-      <c r="N74" s="56" t="n"/>
-      <c r="O74" s="56" t="n"/>
-      <c r="P74" s="56" t="n"/>
-    </row>
-    <row r="75" ht="22" customHeight="1" s="19">
-      <c r="A75" s="59" t="inlineStr">
-        <is>
-          <t>Verlierer HF1</t>
-        </is>
-      </c>
-      <c r="B75" s="59" t="inlineStr"/>
-      <c r="C75" s="66" t="n"/>
-      <c r="D75" s="66" t="n"/>
-      <c r="E75" s="66" t="n"/>
-      <c r="F75" s="66" t="n"/>
-      <c r="G75" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="H75" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="I75" s="65" t="n"/>
-      <c r="J75" s="65" t="n"/>
-      <c r="K75" s="56" t="n"/>
-      <c r="L75" s="56" t="n"/>
-      <c r="M75" s="56" t="n"/>
-      <c r="N75" s="56" t="n"/>
-      <c r="O75" s="56" t="n"/>
-      <c r="P75" s="56" t="n"/>
-    </row>
-    <row r="76" ht="22" customHeight="1" s="19">
-      <c r="A76" s="59" t="n"/>
-      <c r="B76" s="59" t="n"/>
-      <c r="C76" s="66" t="n"/>
-      <c r="D76" s="66" t="n"/>
-      <c r="E76" s="66" t="n"/>
-      <c r="F76" s="66" t="n"/>
-      <c r="G76" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="H76" s="60" t="n"/>
-      <c r="I76" s="65">
-        <f>IF(OR(I75="",G78=""),"",IF(I75&gt;G78,2,IF(I75&lt;G78,0,1)))</f>
-        <v/>
-      </c>
-      <c r="J76" s="65" t="n"/>
-      <c r="K76" s="56" t="n"/>
-      <c r="L76" s="56" t="n"/>
-      <c r="M76" s="56" t="n"/>
-      <c r="N76" s="56" t="n"/>
-      <c r="O76" s="56" t="n"/>
-      <c r="P76" s="56" t="n"/>
-    </row>
-    <row r="77" ht="22" customHeight="1" s="19">
-      <c r="A77" s="59" t="n"/>
-      <c r="B77" s="59" t="n"/>
-      <c r="C77" s="66" t="n"/>
-      <c r="D77" s="66" t="n"/>
-      <c r="E77" s="66" t="n"/>
-      <c r="F77" s="66" t="n"/>
-      <c r="G77" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="H77" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="I77" s="65">
-        <f>IF(J75&gt;0,TRUNC(I75/J75,3),"")</f>
-        <v/>
-      </c>
-      <c r="J77" s="65" t="n"/>
-      <c r="K77" s="56" t="n"/>
-      <c r="L77" s="56" t="n"/>
-      <c r="M77" s="56" t="n"/>
-      <c r="N77" s="56" t="n"/>
-      <c r="O77" s="56" t="n"/>
-      <c r="P77" s="56" t="n"/>
-    </row>
-    <row r="78" ht="22" customHeight="1" s="19">
-      <c r="A78" s="59" t="inlineStr">
-        <is>
-          <t>Verlierer HF2</t>
-        </is>
-      </c>
-      <c r="B78" s="59" t="inlineStr"/>
-      <c r="C78" s="66" t="n"/>
-      <c r="D78" s="66" t="n"/>
-      <c r="E78" s="66" t="n"/>
-      <c r="F78" s="66" t="n"/>
-      <c r="G78" s="65" t="n"/>
-      <c r="H78" s="65" t="n"/>
-      <c r="I78" s="60" t="inlineStr">
-        <is>
-          <t>Bälle</t>
-        </is>
-      </c>
-      <c r="J78" s="60" t="inlineStr">
-        <is>
-          <t>Aufn.</t>
-        </is>
-      </c>
-      <c r="K78" s="56" t="n"/>
-      <c r="L78" s="56" t="n"/>
-      <c r="M78" s="56" t="n"/>
-      <c r="N78" s="56" t="n"/>
-      <c r="O78" s="56" t="n"/>
-      <c r="P78" s="56" t="n"/>
-    </row>
-    <row r="79" ht="22" customHeight="1" s="19">
-      <c r="A79" s="59" t="n"/>
-      <c r="B79" s="59" t="n"/>
-      <c r="C79" s="66" t="n"/>
-      <c r="D79" s="66" t="n"/>
-      <c r="E79" s="66" t="n"/>
-      <c r="F79" s="66" t="n"/>
-      <c r="G79" s="65">
-        <f>IF(OR(G78="",I75=""),"",IF(G78&gt;I75,2,IF(G78&lt;I75,0,1)))</f>
-        <v/>
-      </c>
-      <c r="H79" s="65" t="n"/>
-      <c r="I79" s="60" t="inlineStr">
-        <is>
-          <t>Partiepunkte</t>
-        </is>
-      </c>
-      <c r="J79" s="60" t="n"/>
-      <c r="K79" s="56" t="n"/>
-      <c r="L79" s="56" t="n"/>
-      <c r="M79" s="56" t="n"/>
-      <c r="N79" s="56" t="n"/>
-      <c r="O79" s="56" t="n"/>
-      <c r="P79" s="56" t="n"/>
-    </row>
-    <row r="80" ht="22" customHeight="1" s="19">
-      <c r="A80" s="59" t="n"/>
-      <c r="B80" s="59" t="n"/>
-      <c r="C80" s="66" t="n"/>
-      <c r="D80" s="66" t="n"/>
-      <c r="E80" s="66" t="n"/>
-      <c r="F80" s="66" t="n"/>
-      <c r="G80" s="65">
-        <f>IF(H78&gt;0,TRUNC(G78/H78,3),"")</f>
-        <v/>
-      </c>
-      <c r="H80" s="65" t="n"/>
-      <c r="I80" s="60" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="J80" s="60" t="inlineStr">
-        <is>
-          <t>HS</t>
-        </is>
-      </c>
-      <c r="K80" s="56" t="n"/>
-      <c r="L80" s="56" t="n"/>
-      <c r="M80" s="56" t="n"/>
-      <c r="N80" s="56" t="n"/>
-      <c r="O80" s="56" t="n"/>
-      <c r="P80" s="56" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="56" t="n"/>
-      <c r="B81" s="56" t="n"/>
-      <c r="C81" s="56" t="n"/>
-      <c r="D81" s="56" t="n"/>
-      <c r="E81" s="56" t="n"/>
-      <c r="F81" s="56" t="n"/>
-      <c r="G81" s="56" t="n"/>
-      <c r="H81" s="56" t="n"/>
-      <c r="I81" s="56" t="n"/>
-      <c r="J81" s="56" t="n"/>
-      <c r="K81" s="56" t="n"/>
-      <c r="L81" s="56" t="n"/>
-      <c r="M81" s="56" t="n"/>
-      <c r="N81" s="56" t="n"/>
-      <c r="O81" s="56" t="n"/>
-      <c r="P81" s="56" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="56" t="n"/>
-      <c r="B82" s="56" t="n"/>
-      <c r="C82" s="56" t="n"/>
-      <c r="D82" s="56" t="n"/>
-      <c r="E82" s="56" t="n"/>
-      <c r="F82" s="56" t="n"/>
-      <c r="G82" s="56" t="n"/>
-      <c r="H82" s="56" t="n"/>
-      <c r="I82" s="56" t="n"/>
-      <c r="J82" s="56" t="n"/>
-      <c r="K82" s="56" t="n"/>
-      <c r="L82" s="56" t="n"/>
-      <c r="M82" s="56" t="n"/>
-      <c r="N82" s="56" t="n"/>
-      <c r="O82" s="56" t="n"/>
-      <c r="P82" s="56" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="56" t="n"/>
-      <c r="B83" s="56" t="n"/>
-      <c r="C83" s="56" t="n"/>
-      <c r="D83" s="56" t="n"/>
-      <c r="E83" s="56" t="n"/>
-      <c r="F83" s="56" t="n"/>
-      <c r="G83" s="56" t="n"/>
-      <c r="H83" s="56" t="n"/>
-      <c r="I83" s="56" t="n"/>
-      <c r="J83" s="56" t="n"/>
-      <c r="K83" s="56" t="n"/>
-      <c r="L83" s="56" t="n"/>
-      <c r="M83" s="56" t="n"/>
-      <c r="N83" s="56" t="n"/>
-      <c r="O83" s="56" t="n"/>
-      <c r="P83" s="56" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="56" t="n"/>
-      <c r="B84" s="56" t="n"/>
-      <c r="C84" s="56" t="n"/>
-      <c r="D84" s="56" t="n"/>
-      <c r="E84" s="56" t="n"/>
-      <c r="F84" s="56" t="n"/>
-      <c r="G84" s="56" t="n"/>
-      <c r="H84" s="56" t="n"/>
-      <c r="I84" s="56" t="n"/>
-      <c r="J84" s="56" t="n"/>
-      <c r="K84" s="56" t="n"/>
-      <c r="L84" s="56" t="n"/>
-      <c r="M84" s="56" t="n"/>
-      <c r="N84" s="56" t="n"/>
-      <c r="O84" s="56" t="n"/>
-      <c r="P84" s="56" t="n"/>
-    </row>
+    <row r="37" ht="24" customHeight="1" s="19"/>
+    <row r="38" ht="24" customHeight="1" s="19"/>
+    <row r="39" ht="22" customHeight="1" s="19"/>
+    <row r="40" ht="22" customHeight="1" s="19"/>
+    <row r="41" ht="22" customHeight="1" s="19"/>
+    <row r="42" ht="22" customHeight="1" s="19"/>
+    <row r="43" ht="22" customHeight="1" s="19"/>
+    <row r="44" ht="22" customHeight="1" s="19"/>
+    <row r="45" ht="22" customHeight="1" s="19"/>
+    <row r="46" ht="22" customHeight="1" s="19"/>
+    <row r="47" ht="22" customHeight="1" s="19"/>
+    <row r="48" ht="22" customHeight="1" s="19"/>
+    <row r="49" ht="22" customHeight="1" s="19"/>
+    <row r="50" ht="22" customHeight="1" s="19"/>
+    <row r="52" ht="24" customHeight="1" s="19"/>
+    <row r="53" ht="24" customHeight="1" s="19"/>
+    <row r="54" ht="22" customHeight="1" s="19"/>
+    <row r="55" ht="22" customHeight="1" s="19"/>
+    <row r="56" ht="22" customHeight="1" s="19"/>
+    <row r="57" ht="22" customHeight="1" s="19"/>
+    <row r="58" ht="22" customHeight="1" s="19"/>
+    <row r="59" ht="22" customHeight="1" s="19"/>
+    <row r="60" ht="22" customHeight="1" s="19"/>
+    <row r="61" ht="22" customHeight="1" s="19"/>
+    <row r="62" ht="22" customHeight="1" s="19"/>
+    <row r="63" ht="22" customHeight="1" s="19"/>
+    <row r="64" ht="22" customHeight="1" s="19"/>
+    <row r="65" ht="22" customHeight="1" s="19"/>
+    <row r="67" ht="24" customHeight="1" s="19"/>
+    <row r="68" ht="24" customHeight="1" s="19"/>
+    <row r="69" ht="22" customHeight="1" s="19"/>
+    <row r="70" ht="22" customHeight="1" s="19"/>
+    <row r="71" ht="22" customHeight="1" s="19"/>
+    <row r="72" ht="22" customHeight="1" s="19"/>
+    <row r="73" ht="22" customHeight="1" s="19"/>
+    <row r="74" ht="22" customHeight="1" s="19"/>
+    <row r="75" ht="22" customHeight="1" s="19"/>
+    <row r="76" ht="22" customHeight="1" s="19"/>
+    <row r="77" ht="22" customHeight="1" s="19"/>
+    <row r="78" ht="22" customHeight="1" s="19"/>
+    <row r="79" ht="22" customHeight="1" s="19"/>
+    <row r="80" ht="22" customHeight="1" s="19"/>
   </sheetData>
-  <mergeCells count="186">
+  <mergeCells count="99">
     <mergeCell ref="O31:O33"/>
     <mergeCell ref="M12:M14"/>
-    <mergeCell ref="A57:A59"/>
     <mergeCell ref="F29:G29"/>
     <mergeCell ref="O12:O14"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="J25:J27"/>
     <mergeCell ref="L25:L27"/>
-    <mergeCell ref="A72:A74"/>
     <mergeCell ref="N28:N30"/>
-    <mergeCell ref="C45:D47"/>
     <mergeCell ref="N6:N8"/>
-    <mergeCell ref="A52:J52"/>
     <mergeCell ref="L9:L11"/>
-    <mergeCell ref="G39:H41"/>
-    <mergeCell ref="E48:F50"/>
     <mergeCell ref="N9:N11"/>
-    <mergeCell ref="C73:D73"/>
-    <mergeCell ref="E73:F73"/>
-    <mergeCell ref="B45:B47"/>
     <mergeCell ref="B21:C21"/>
-    <mergeCell ref="G57:H59"/>
-    <mergeCell ref="I57:J59"/>
-    <mergeCell ref="I76:J76"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="C43:D43"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="C60:D62"/>
     <mergeCell ref="F23:G23"/>
-    <mergeCell ref="B72:B74"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="M6:M8"/>
-    <mergeCell ref="B57:B59"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="L15:L17"/>
     <mergeCell ref="M25:M27"/>
     <mergeCell ref="O25:O27"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="H23:I23"/>
-    <mergeCell ref="E53:F53"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="A42:A44"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
-    <mergeCell ref="E55:F55"/>
     <mergeCell ref="F10:G10"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G61:H61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="I54:J56"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="A67:J67"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="C40:D40"/>
     <mergeCell ref="A31:A33"/>
     <mergeCell ref="K15:K17"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C75:D77"/>
-    <mergeCell ref="E78:F80"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="I72:J74"/>
     <mergeCell ref="A20:O20"/>
-    <mergeCell ref="B75:B77"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="I69:J71"/>
-    <mergeCell ref="A60:A62"/>
     <mergeCell ref="O15:O17"/>
-    <mergeCell ref="A69:A71"/>
     <mergeCell ref="J28:J30"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="L28:L30"/>
-    <mergeCell ref="A54:A56"/>
     <mergeCell ref="N22:N24"/>
-    <mergeCell ref="C48:D50"/>
     <mergeCell ref="L12:L14"/>
-    <mergeCell ref="B39:B41"/>
     <mergeCell ref="N12:N14"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="G76:H76"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="A25:A27"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="K12:K14"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="C68:D68"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="A63:A65"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="F21:G21"/>
     <mergeCell ref="K28:K30"/>
     <mergeCell ref="K6:K8"/>
     <mergeCell ref="H21:I21"/>
-    <mergeCell ref="G69:H71"/>
     <mergeCell ref="A28:A30"/>
     <mergeCell ref="K25:K27"/>
-    <mergeCell ref="B63:B65"/>
     <mergeCell ref="O28:O30"/>
     <mergeCell ref="O6:O8"/>
     <mergeCell ref="K9:K11"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="O9:O11"/>
-    <mergeCell ref="A45:A47"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="N25:N27"/>
-    <mergeCell ref="E45:F47"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="I39:J41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="G54:H56"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="G79:H79"/>
-    <mergeCell ref="I79:J79"/>
     <mergeCell ref="J9:J11"/>
-    <mergeCell ref="C38:D38"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D5:E5"/>
-    <mergeCell ref="C78:D80"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="G72:H74"/>
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="H29:I29"/>
-    <mergeCell ref="I49:J49"/>
     <mergeCell ref="J22:J24"/>
     <mergeCell ref="L22:L24"/>
     <mergeCell ref="J31:J33"/>
-    <mergeCell ref="E63:F65"/>
     <mergeCell ref="L31:L33"/>
     <mergeCell ref="D21:E21"/>
-    <mergeCell ref="B54:B56"/>
     <mergeCell ref="N31:N33"/>
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="L6:L8"/>
-    <mergeCell ref="G42:H44"/>
-    <mergeCell ref="E60:F62"/>
     <mergeCell ref="N15:N17"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="C63:D65"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G53:H53"/>
     <mergeCell ref="F32:G32"/>
-    <mergeCell ref="I53:J53"/>
     <mergeCell ref="F26:G26"/>
     <mergeCell ref="A4:O4"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A39:A41"/>
     <mergeCell ref="D16:E16"/>
-    <mergeCell ref="I68:J68"/>
-    <mergeCell ref="A48:A50"/>
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="I42:J44"/>
-    <mergeCell ref="A78:A80"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A75:A77"/>
     <mergeCell ref="K22:K24"/>
-    <mergeCell ref="I38:J38"/>
     <mergeCell ref="M22:M24"/>
     <mergeCell ref="K31:K33"/>
     <mergeCell ref="M31:M33"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="B69:B71"/>
-    <mergeCell ref="E75:F77"/>
     <mergeCell ref="M15:M17"/>
     <mergeCell ref="M28:M30"/>
     <mergeCell ref="O22:O24"/>
@@ -4569,35 +3414,35 @@
         <v>1</v>
       </c>
       <c r="D14" s="15">
-        <f>IF(Tableau!B39="","",Tableau!B39)</f>
+        <f>IF(Finalrunde!A6="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A6,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E14" s="15">
-        <f>IF(Tableau!B42="","",Tableau!B42)</f>
+        <f>IF(Finalrunde!A9="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A9,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>IF(Tableau!E39="","",Tableau!E39)</f>
+        <f>IF(Finalrunde!D6="","",Finalrunde!D6)</f>
         <v/>
       </c>
       <c r="G14" s="15">
-        <f>IF(Tableau!C42="","",Tableau!C42)</f>
+        <f>IF(Finalrunde!B9="","",Finalrunde!B9)</f>
         <v/>
       </c>
       <c r="H14" s="15">
-        <f>IF(Tableau!F39="","",Tableau!F39)</f>
+        <f>IF(Finalrunde!E6="","",Finalrunde!E6)</f>
         <v/>
       </c>
       <c r="I14" s="15">
-        <f>IF(Tableau!D42="","",Tableau!D42)</f>
+        <f>IF(Finalrunde!C9="","",Finalrunde!C9)</f>
         <v/>
       </c>
       <c r="J14" s="15">
-        <f>IF(Tableau!F41="","",Tableau!F41)</f>
+        <f>IF(Finalrunde!E8="","",Finalrunde!E8)</f>
         <v/>
       </c>
       <c r="K14" s="15">
-        <f>IF(Tableau!D44="","",Tableau!D44)</f>
+        <f>IF(Finalrunde!C11="","",Finalrunde!C11)</f>
         <v/>
       </c>
       <c r="L14" s="15">
@@ -4619,35 +3464,35 @@
         <v>1</v>
       </c>
       <c r="D15" s="15">
-        <f>IF(Tableau!B45="","",Tableau!B45)</f>
+        <f>IF(Finalrunde!A12="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A12,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E15" s="15">
-        <f>IF(Tableau!B48="","",Tableau!B48)</f>
+        <f>IF(Finalrunde!A15="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A15,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F15" s="15">
-        <f>IF(Tableau!I45="","",Tableau!I45)</f>
+        <f>IF(Finalrunde!H12="","",Finalrunde!H12)</f>
         <v/>
       </c>
       <c r="G15" s="15">
-        <f>IF(Tableau!G48="","",Tableau!G48)</f>
+        <f>IF(Finalrunde!F15="","",Finalrunde!F15)</f>
         <v/>
       </c>
       <c r="H15" s="15">
-        <f>IF(Tableau!J45="","",Tableau!J45)</f>
+        <f>IF(Finalrunde!I12="","",Finalrunde!I12)</f>
         <v/>
       </c>
       <c r="I15" s="15">
-        <f>IF(Tableau!H48="","",Tableau!H48)</f>
+        <f>IF(Finalrunde!G15="","",Finalrunde!G15)</f>
         <v/>
       </c>
       <c r="J15" s="15">
-        <f>IF(Tableau!J47="","",Tableau!J47)</f>
+        <f>IF(Finalrunde!I14="","",Finalrunde!I14)</f>
         <v/>
       </c>
       <c r="K15" s="15">
-        <f>IF(Tableau!H50="","",Tableau!H50)</f>
+        <f>IF(Finalrunde!G17="","",Finalrunde!G17)</f>
         <v/>
       </c>
       <c r="L15" s="15">
@@ -4669,35 +3514,35 @@
         <v>1</v>
       </c>
       <c r="D16" s="15">
-        <f>IF(Tableau!B54="","",Tableau!B54)</f>
+        <f>IF(Finalrunde!A21="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A21,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E16" s="15">
-        <f>IF(Tableau!B57="","",Tableau!B57)</f>
+        <f>IF(Finalrunde!A24="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A24,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>IF(Tableau!E54="","",Tableau!E54)</f>
+        <f>IF(Finalrunde!D21="","",Finalrunde!D21)</f>
         <v/>
       </c>
       <c r="G16" s="15">
-        <f>IF(Tableau!C57="","",Tableau!C57)</f>
+        <f>IF(Finalrunde!B24="","",Finalrunde!B24)</f>
         <v/>
       </c>
       <c r="H16" s="15">
-        <f>IF(Tableau!F54="","",Tableau!F54)</f>
+        <f>IF(Finalrunde!E21="","",Finalrunde!E21)</f>
         <v/>
       </c>
       <c r="I16" s="15">
-        <f>IF(Tableau!D57="","",Tableau!D57)</f>
+        <f>IF(Finalrunde!C24="","",Finalrunde!C24)</f>
         <v/>
       </c>
       <c r="J16" s="15">
-        <f>IF(Tableau!F56="","",Tableau!F56)</f>
+        <f>IF(Finalrunde!E23="","",Finalrunde!E23)</f>
         <v/>
       </c>
       <c r="K16" s="15">
-        <f>IF(Tableau!D59="","",Tableau!D59)</f>
+        <f>IF(Finalrunde!C26="","",Finalrunde!C26)</f>
         <v/>
       </c>
       <c r="L16" s="15">
@@ -4719,35 +3564,35 @@
         <v>1</v>
       </c>
       <c r="D17" s="15">
-        <f>IF(Tableau!B60="","",Tableau!B60)</f>
+        <f>IF(Finalrunde!A27="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A27,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E17" s="15">
-        <f>IF(Tableau!B63="","",Tableau!B63)</f>
+        <f>IF(Finalrunde!A30="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A30,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F17" s="15">
-        <f>IF(Tableau!I60="","",Tableau!I60)</f>
+        <f>IF(Finalrunde!H27="","",Finalrunde!H27)</f>
         <v/>
       </c>
       <c r="G17" s="15">
-        <f>IF(Tableau!G63="","",Tableau!G63)</f>
+        <f>IF(Finalrunde!F30="","",Finalrunde!F30)</f>
         <v/>
       </c>
       <c r="H17" s="15">
-        <f>IF(Tableau!J60="","",Tableau!J60)</f>
+        <f>IF(Finalrunde!I27="","",Finalrunde!I27)</f>
         <v/>
       </c>
       <c r="I17" s="15">
-        <f>IF(Tableau!H63="","",Tableau!H63)</f>
+        <f>IF(Finalrunde!G30="","",Finalrunde!G30)</f>
         <v/>
       </c>
       <c r="J17" s="15">
-        <f>IF(Tableau!J62="","",Tableau!J62)</f>
+        <f>IF(Finalrunde!I29="","",Finalrunde!I29)</f>
         <v/>
       </c>
       <c r="K17" s="15">
-        <f>IF(Tableau!H65="","",Tableau!H65)</f>
+        <f>IF(Finalrunde!G32="","",Finalrunde!G32)</f>
         <v/>
       </c>
       <c r="L17" s="15">
@@ -4769,35 +3614,35 @@
         <v>1</v>
       </c>
       <c r="D18" s="15">
-        <f>IF(Tableau!B69="","",Tableau!B69)</f>
+        <f>IF(Finalrunde!A36="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A36,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E18" s="15">
-        <f>IF(Tableau!B72="","",Tableau!B72)</f>
+        <f>IF(Finalrunde!A39="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A39,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F18" s="15">
-        <f>IF(Tableau!E69="","",Tableau!E69)</f>
+        <f>IF(Finalrunde!D36="","",Finalrunde!D36)</f>
         <v/>
       </c>
       <c r="G18" s="15">
-        <f>IF(Tableau!C72="","",Tableau!C72)</f>
+        <f>IF(Finalrunde!B39="","",Finalrunde!B39)</f>
         <v/>
       </c>
       <c r="H18" s="15">
-        <f>IF(Tableau!F69="","",Tableau!F69)</f>
+        <f>IF(Finalrunde!E36="","",Finalrunde!E36)</f>
         <v/>
       </c>
       <c r="I18" s="15">
-        <f>IF(Tableau!D72="","",Tableau!D72)</f>
+        <f>IF(Finalrunde!C39="","",Finalrunde!C39)</f>
         <v/>
       </c>
       <c r="J18" s="15">
-        <f>IF(Tableau!F71="","",Tableau!F71)</f>
+        <f>IF(Finalrunde!E38="","",Finalrunde!E38)</f>
         <v/>
       </c>
       <c r="K18" s="15">
-        <f>IF(Tableau!D74="","",Tableau!D74)</f>
+        <f>IF(Finalrunde!C41="","",Finalrunde!C41)</f>
         <v/>
       </c>
       <c r="L18" s="15">
@@ -4819,35 +3664,35 @@
         <v>1</v>
       </c>
       <c r="D19" s="15">
-        <f>IF(Tableau!B75="","",Tableau!B75)</f>
+        <f>IF(Finalrunde!A42="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A42,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="E19" s="15">
-        <f>IF(Tableau!B78="","",Tableau!B78)</f>
+        <f>IF(Finalrunde!A45="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(Finalrunde!A45,Teilnehmer!$B$2:$B$9,0)),""))</f>
         <v/>
       </c>
       <c r="F19" s="15">
-        <f>IF(Tableau!I75="","",Tableau!I75)</f>
+        <f>IF(Finalrunde!H42="","",Finalrunde!H42)</f>
         <v/>
       </c>
       <c r="G19" s="15">
-        <f>IF(Tableau!G78="","",Tableau!G78)</f>
+        <f>IF(Finalrunde!F45="","",Finalrunde!F45)</f>
         <v/>
       </c>
       <c r="H19" s="15">
-        <f>IF(Tableau!J75="","",Tableau!J75)</f>
+        <f>IF(Finalrunde!I42="","",Finalrunde!I42)</f>
         <v/>
       </c>
       <c r="I19" s="15">
-        <f>IF(Tableau!H78="","",Tableau!H78)</f>
+        <f>IF(Finalrunde!G45="","",Finalrunde!G45)</f>
         <v/>
       </c>
       <c r="J19" s="15">
-        <f>IF(Tableau!J77="","",Tableau!J77)</f>
+        <f>IF(Finalrunde!I44="","",Finalrunde!I44)</f>
         <v/>
       </c>
       <c r="K19" s="15">
-        <f>IF(Tableau!H80="","",Tableau!H80)</f>
+        <f>IF(Finalrunde!G47="","",Finalrunde!G47)</f>
         <v/>
       </c>
       <c r="L19" s="15">
@@ -4882,4 +3727,1020 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="19" min="1" max="1"/>
+    <col width="11" customWidth="1" style="19" min="2" max="2"/>
+    <col width="11" customWidth="1" style="19" min="3" max="3"/>
+    <col width="11" customWidth="1" style="19" min="4" max="4"/>
+    <col width="11" customWidth="1" style="19" min="5" max="5"/>
+    <col width="11" customWidth="1" style="19" min="6" max="6"/>
+    <col width="11" customWidth="1" style="19" min="7" max="7"/>
+    <col width="11" customWidth="1" style="19" min="8" max="8"/>
+    <col width="11" customWidth="1" style="19" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="19">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>Final- und Platzierungsspiele</t>
+        </is>
+      </c>
+      <c r="B1" s="71" t="n"/>
+      <c r="C1" s="71" t="n"/>
+      <c r="D1" s="71" t="n"/>
+      <c r="E1" s="71" t="n"/>
+      <c r="F1" s="71" t="n"/>
+      <c r="G1" s="71" t="n"/>
+      <c r="H1" s="71" t="n"/>
+      <c r="I1" s="71" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="19">
+      <c r="A2" s="68" t="inlineStr">
+        <is>
+          <t>Die Spieler werden aus den Gruppenplatzierungen ermittelt. Namen aktualisieren sich nach Eingabe der Gruppenergebnisse.</t>
+        </is>
+      </c>
+      <c r="B2" s="72" t="n"/>
+      <c r="C2" s="72" t="n"/>
+      <c r="D2" s="72" t="n"/>
+      <c r="E2" s="72" t="n"/>
+      <c r="F2" s="72" t="n"/>
+      <c r="G2" s="72" t="n"/>
+      <c r="H2" s="72" t="n"/>
+      <c r="I2" s="72" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1" s="19">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>Halbfinale</t>
+        </is>
+      </c>
+      <c r="B4" s="73" t="n"/>
+      <c r="C4" s="73" t="n"/>
+      <c r="D4" s="73" t="n"/>
+      <c r="E4" s="73" t="n"/>
+      <c r="F4" s="73" t="n"/>
+      <c r="G4" s="73" t="n"/>
+      <c r="H4" s="73" t="n"/>
+      <c r="I4" s="73" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="19">
+      <c r="A5" s="57" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="B5" s="57" t="inlineStr">
+        <is>
+          <t>1. Gruppe 1</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="n"/>
+      <c r="D5" s="57" t="inlineStr">
+        <is>
+          <t>2. Gruppe 2</t>
+        </is>
+      </c>
+      <c r="E5" s="74" t="n"/>
+      <c r="F5" s="57" t="inlineStr">
+        <is>
+          <t>1. Gruppe 2</t>
+        </is>
+      </c>
+      <c r="G5" s="74" t="n"/>
+      <c r="H5" s="57" t="inlineStr">
+        <is>
+          <t>2. Gruppe 1</t>
+        </is>
+      </c>
+      <c r="I5" s="74" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="19">
+      <c r="A6" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$6:$A$15,MATCH(1,'Tableau'!$O$6:$O$15,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="D6" s="65" t="n"/>
+      <c r="E6" s="65" t="n"/>
+      <c r="F6" s="66" t="n"/>
+      <c r="G6" s="75" t="n"/>
+      <c r="H6" s="66" t="n"/>
+      <c r="I6" s="75" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="19">
+      <c r="A7" s="76" t="n"/>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="C7" s="74" t="n"/>
+      <c r="D7" s="65">
+        <f>IF(OR(D6="",B9=""),"",IF(D6&gt;B9,2,IF(D6&lt;B9,0,1)))</f>
+        <v/>
+      </c>
+      <c r="E7" s="74" t="n"/>
+      <c r="F7" s="77" t="n"/>
+      <c r="G7" s="78" t="n"/>
+      <c r="H7" s="77" t="n"/>
+      <c r="I7" s="78" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" s="19">
+      <c r="A8" s="79" t="n"/>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="D8" s="65">
+        <f>IF(E6&gt;0,TRUNC(D6/E6,3),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="65" t="n"/>
+      <c r="F8" s="80" t="n"/>
+      <c r="G8" s="81" t="n"/>
+      <c r="H8" s="80" t="n"/>
+      <c r="I8" s="81" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" s="19">
+      <c r="A9" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$22:$A$31,MATCH(2,'Tableau'!$O$22:$O$31,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B9" s="65" t="n"/>
+      <c r="C9" s="65" t="n"/>
+      <c r="D9" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="E9" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="F9" s="66" t="n"/>
+      <c r="G9" s="75" t="n"/>
+      <c r="H9" s="66" t="n"/>
+      <c r="I9" s="75" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="19">
+      <c r="A10" s="76" t="n"/>
+      <c r="B10" s="65">
+        <f>IF(OR(B9="",D6=""),"",IF(B9&gt;D6,2,IF(B9&lt;D6,0,1)))</f>
+        <v/>
+      </c>
+      <c r="C10" s="74" t="n"/>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="77" t="n"/>
+      <c r="G10" s="78" t="n"/>
+      <c r="H10" s="77" t="n"/>
+      <c r="I10" s="78" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1" s="19">
+      <c r="A11" s="79" t="n"/>
+      <c r="B11" s="65">
+        <f>IF(C9&gt;0,TRUNC(B9/C9,3),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="65" t="n"/>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="E11" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="F11" s="80" t="n"/>
+      <c r="G11" s="81" t="n"/>
+      <c r="H11" s="80" t="n"/>
+      <c r="I11" s="81" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1" s="19">
+      <c r="A12" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$22:$A$31,MATCH(1,'Tableau'!$O$22:$O$31,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="75" t="n"/>
+      <c r="D12" s="66" t="n"/>
+      <c r="E12" s="75" t="n"/>
+      <c r="F12" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="G12" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="H12" s="65" t="n"/>
+      <c r="I12" s="65" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="19">
+      <c r="A13" s="76" t="n"/>
+      <c r="B13" s="77" t="n"/>
+      <c r="C13" s="78" t="n"/>
+      <c r="D13" s="77" t="n"/>
+      <c r="E13" s="78" t="n"/>
+      <c r="F13" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="G13" s="74" t="n"/>
+      <c r="H13" s="65">
+        <f>IF(OR(H12="",F15=""),"",IF(H12&gt;F15,2,IF(H12&lt;F15,0,1)))</f>
+        <v/>
+      </c>
+      <c r="I13" s="74" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="19">
+      <c r="A14" s="79" t="n"/>
+      <c r="B14" s="80" t="n"/>
+      <c r="C14" s="81" t="n"/>
+      <c r="D14" s="80" t="n"/>
+      <c r="E14" s="81" t="n"/>
+      <c r="F14" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G14" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="H14" s="65">
+        <f>IF(I12&gt;0,TRUNC(H12/I12,3),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="65" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1" s="19">
+      <c r="A15" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$6:$A$15,MATCH(2,'Tableau'!$O$6:$O$15,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B15" s="66" t="n"/>
+      <c r="C15" s="75" t="n"/>
+      <c r="D15" s="66" t="n"/>
+      <c r="E15" s="75" t="n"/>
+      <c r="F15" s="65" t="n"/>
+      <c r="G15" s="65" t="n"/>
+      <c r="H15" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="I15" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="19">
+      <c r="A16" s="76" t="n"/>
+      <c r="B16" s="77" t="n"/>
+      <c r="C16" s="78" t="n"/>
+      <c r="D16" s="77" t="n"/>
+      <c r="E16" s="78" t="n"/>
+      <c r="F16" s="65">
+        <f>IF(OR(F15="",H12=""),"",IF(F15&gt;H12,2,IF(F15&lt;H12,0,1)))</f>
+        <v/>
+      </c>
+      <c r="G16" s="74" t="n"/>
+      <c r="H16" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="I16" s="74" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="19">
+      <c r="A17" s="79" t="n"/>
+      <c r="B17" s="80" t="n"/>
+      <c r="C17" s="81" t="n"/>
+      <c r="D17" s="80" t="n"/>
+      <c r="E17" s="81" t="n"/>
+      <c r="F17" s="65">
+        <f>IF(G15&gt;0,TRUNC(F15/G15,3),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="65" t="n"/>
+      <c r="H17" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="I17" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1" s="19">
+      <c r="A19" s="69" t="inlineStr">
+        <is>
+          <t>Platzierung 5-8</t>
+        </is>
+      </c>
+      <c r="B19" s="73" t="n"/>
+      <c r="C19" s="73" t="n"/>
+      <c r="D19" s="73" t="n"/>
+      <c r="E19" s="73" t="n"/>
+      <c r="F19" s="73" t="n"/>
+      <c r="G19" s="73" t="n"/>
+      <c r="H19" s="73" t="n"/>
+      <c r="I19" s="73" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="19">
+      <c r="A20" s="57" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="B20" s="57" t="inlineStr">
+        <is>
+          <t>3. Gruppe 1</t>
+        </is>
+      </c>
+      <c r="C20" s="74" t="n"/>
+      <c r="D20" s="57" t="inlineStr">
+        <is>
+          <t>3. Gruppe 2</t>
+        </is>
+      </c>
+      <c r="E20" s="74" t="n"/>
+      <c r="F20" s="57" t="inlineStr">
+        <is>
+          <t>4. Gruppe 1</t>
+        </is>
+      </c>
+      <c r="G20" s="74" t="n"/>
+      <c r="H20" s="57" t="inlineStr">
+        <is>
+          <t>4. Gruppe 2</t>
+        </is>
+      </c>
+      <c r="I20" s="74" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="19">
+      <c r="A21" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$6:$A$15,MATCH(3,'Tableau'!$O$6:$O$15,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B21" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="D21" s="65" t="n"/>
+      <c r="E21" s="65" t="n"/>
+      <c r="F21" s="66" t="n"/>
+      <c r="G21" s="75" t="n"/>
+      <c r="H21" s="66" t="n"/>
+      <c r="I21" s="75" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" s="19">
+      <c r="A22" s="76" t="n"/>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="C22" s="74" t="n"/>
+      <c r="D22" s="65">
+        <f>IF(OR(D21="",B24=""),"",IF(D21&gt;B24,2,IF(D21&lt;B24,0,1)))</f>
+        <v/>
+      </c>
+      <c r="E22" s="74" t="n"/>
+      <c r="F22" s="77" t="n"/>
+      <c r="G22" s="78" t="n"/>
+      <c r="H22" s="77" t="n"/>
+      <c r="I22" s="78" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="19">
+      <c r="A23" s="79" t="n"/>
+      <c r="B23" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="C23" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="D23" s="65">
+        <f>IF(E21&gt;0,TRUNC(D21/E21,3),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="65" t="n"/>
+      <c r="F23" s="80" t="n"/>
+      <c r="G23" s="81" t="n"/>
+      <c r="H23" s="80" t="n"/>
+      <c r="I23" s="81" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" s="19">
+      <c r="A24" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$22:$A$31,MATCH(3,'Tableau'!$O$22:$O$31,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B24" s="65" t="n"/>
+      <c r="C24" s="65" t="n"/>
+      <c r="D24" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="E24" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="F24" s="66" t="n"/>
+      <c r="G24" s="75" t="n"/>
+      <c r="H24" s="66" t="n"/>
+      <c r="I24" s="75" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="19">
+      <c r="A25" s="76" t="n"/>
+      <c r="B25" s="65">
+        <f>IF(OR(B24="",D21=""),"",IF(B24&gt;D21,2,IF(B24&lt;D21,0,1)))</f>
+        <v/>
+      </c>
+      <c r="C25" s="74" t="n"/>
+      <c r="D25" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="E25" s="74" t="n"/>
+      <c r="F25" s="77" t="n"/>
+      <c r="G25" s="78" t="n"/>
+      <c r="H25" s="77" t="n"/>
+      <c r="I25" s="78" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1" s="19">
+      <c r="A26" s="79" t="n"/>
+      <c r="B26" s="65">
+        <f>IF(C24&gt;0,TRUNC(B24/C24,3),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="65" t="n"/>
+      <c r="D26" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="E26" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="F26" s="80" t="n"/>
+      <c r="G26" s="81" t="n"/>
+      <c r="H26" s="80" t="n"/>
+      <c r="I26" s="81" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="19">
+      <c r="A27" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$6:$A$15,MATCH(4,'Tableau'!$O$6:$O$15,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B27" s="66" t="n"/>
+      <c r="C27" s="75" t="n"/>
+      <c r="D27" s="66" t="n"/>
+      <c r="E27" s="75" t="n"/>
+      <c r="F27" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="G27" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="H27" s="65" t="n"/>
+      <c r="I27" s="65" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1" s="19">
+      <c r="A28" s="76" t="n"/>
+      <c r="B28" s="77" t="n"/>
+      <c r="C28" s="78" t="n"/>
+      <c r="D28" s="77" t="n"/>
+      <c r="E28" s="78" t="n"/>
+      <c r="F28" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="G28" s="74" t="n"/>
+      <c r="H28" s="65">
+        <f>IF(OR(H27="",F30=""),"",IF(H27&gt;F30,2,IF(H27&lt;F30,0,1)))</f>
+        <v/>
+      </c>
+      <c r="I28" s="74" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="19">
+      <c r="A29" s="79" t="n"/>
+      <c r="B29" s="80" t="n"/>
+      <c r="C29" s="81" t="n"/>
+      <c r="D29" s="80" t="n"/>
+      <c r="E29" s="81" t="n"/>
+      <c r="F29" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G29" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="H29" s="65">
+        <f>IF(I27&gt;0,TRUNC(H27/I27,3),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="65" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="19">
+      <c r="A30" s="70">
+        <f>IFERROR(INDEX('Tableau'!$A$22:$A$31,MATCH(4,'Tableau'!$O$22:$O$31,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B30" s="66" t="n"/>
+      <c r="C30" s="75" t="n"/>
+      <c r="D30" s="66" t="n"/>
+      <c r="E30" s="75" t="n"/>
+      <c r="F30" s="65" t="n"/>
+      <c r="G30" s="65" t="n"/>
+      <c r="H30" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="I30" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" s="19">
+      <c r="A31" s="76" t="n"/>
+      <c r="B31" s="77" t="n"/>
+      <c r="C31" s="78" t="n"/>
+      <c r="D31" s="77" t="n"/>
+      <c r="E31" s="78" t="n"/>
+      <c r="F31" s="65">
+        <f>IF(OR(F30="",H27=""),"",IF(F30&gt;H27,2,IF(F30&lt;H27,0,1)))</f>
+        <v/>
+      </c>
+      <c r="G31" s="74" t="n"/>
+      <c r="H31" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="I31" s="74" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="19">
+      <c r="A32" s="79" t="n"/>
+      <c r="B32" s="80" t="n"/>
+      <c r="C32" s="81" t="n"/>
+      <c r="D32" s="80" t="n"/>
+      <c r="E32" s="81" t="n"/>
+      <c r="F32" s="65">
+        <f>IF(G30&gt;0,TRUNC(F30/G30,3),"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="65" t="n"/>
+      <c r="H32" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="I32" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1" s="19">
+      <c r="A34" s="69" t="inlineStr">
+        <is>
+          <t>Endspiele</t>
+        </is>
+      </c>
+      <c r="B34" s="73" t="n"/>
+      <c r="C34" s="73" t="n"/>
+      <c r="D34" s="73" t="n"/>
+      <c r="E34" s="73" t="n"/>
+      <c r="F34" s="73" t="n"/>
+      <c r="G34" s="73" t="n"/>
+      <c r="H34" s="73" t="n"/>
+      <c r="I34" s="73" t="n"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" s="19">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="B35" s="57" t="inlineStr">
+        <is>
+          <t>Sieger HF1</t>
+        </is>
+      </c>
+      <c r="C35" s="74" t="n"/>
+      <c r="D35" s="57" t="inlineStr">
+        <is>
+          <t>Sieger HF2</t>
+        </is>
+      </c>
+      <c r="E35" s="74" t="n"/>
+      <c r="F35" s="57" t="inlineStr">
+        <is>
+          <t>Verlierer HF1</t>
+        </is>
+      </c>
+      <c r="G35" s="74" t="n"/>
+      <c r="H35" s="57" t="inlineStr">
+        <is>
+          <t>Verlierer HF2</t>
+        </is>
+      </c>
+      <c r="I35" s="74" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1" s="19">
+      <c r="A36" s="70">
+        <f>IF(OR(D6="",B9=""),"",IF(D6&gt;B9,A6,IF(B9&gt;D6,A9,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="B36" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="C36" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="D36" s="65" t="n"/>
+      <c r="E36" s="65" t="n"/>
+      <c r="F36" s="66" t="n"/>
+      <c r="G36" s="75" t="n"/>
+      <c r="H36" s="66" t="n"/>
+      <c r="I36" s="75" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1" s="19">
+      <c r="A37" s="76" t="n"/>
+      <c r="B37" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="C37" s="74" t="n"/>
+      <c r="D37" s="65">
+        <f>IF(OR(D36="",B39=""),"",IF(D36&gt;B39,2,IF(D36&lt;B39,0,1)))</f>
+        <v/>
+      </c>
+      <c r="E37" s="74" t="n"/>
+      <c r="F37" s="77" t="n"/>
+      <c r="G37" s="78" t="n"/>
+      <c r="H37" s="77" t="n"/>
+      <c r="I37" s="78" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1" s="19">
+      <c r="A38" s="79" t="n"/>
+      <c r="B38" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="C38" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="D38" s="65">
+        <f>IF(E36&gt;0,TRUNC(D36/E36,3),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="65" t="n"/>
+      <c r="F38" s="80" t="n"/>
+      <c r="G38" s="81" t="n"/>
+      <c r="H38" s="80" t="n"/>
+      <c r="I38" s="81" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1" s="19">
+      <c r="A39" s="70">
+        <f>IF(OR(H12="",F15=""),"",IF(H12&gt;F15,A12,IF(F15&gt;H12,A15,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="B39" s="65" t="n"/>
+      <c r="C39" s="65" t="n"/>
+      <c r="D39" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="E39" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="F39" s="66" t="n"/>
+      <c r="G39" s="75" t="n"/>
+      <c r="H39" s="66" t="n"/>
+      <c r="I39" s="75" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1" s="19">
+      <c r="A40" s="76" t="n"/>
+      <c r="B40" s="65">
+        <f>IF(OR(B39="",D36=""),"",IF(B39&gt;D36,2,IF(B39&lt;D36,0,1)))</f>
+        <v/>
+      </c>
+      <c r="C40" s="74" t="n"/>
+      <c r="D40" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="E40" s="74" t="n"/>
+      <c r="F40" s="77" t="n"/>
+      <c r="G40" s="78" t="n"/>
+      <c r="H40" s="77" t="n"/>
+      <c r="I40" s="78" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1" s="19">
+      <c r="A41" s="79" t="n"/>
+      <c r="B41" s="65">
+        <f>IF(C39&gt;0,TRUNC(B39/C39,3),"")</f>
+        <v/>
+      </c>
+      <c r="C41" s="65" t="n"/>
+      <c r="D41" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="E41" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="F41" s="80" t="n"/>
+      <c r="G41" s="81" t="n"/>
+      <c r="H41" s="80" t="n"/>
+      <c r="I41" s="81" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1" s="19">
+      <c r="A42" s="70">
+        <f>IF(OR(D6="",B9=""),"",IF(D6&lt;B9,A6,IF(B9&lt;D6,A9,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="B42" s="66" t="n"/>
+      <c r="C42" s="75" t="n"/>
+      <c r="D42" s="66" t="n"/>
+      <c r="E42" s="75" t="n"/>
+      <c r="F42" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="G42" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+      <c r="H42" s="65" t="n"/>
+      <c r="I42" s="65" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1" s="19">
+      <c r="A43" s="76" t="n"/>
+      <c r="B43" s="77" t="n"/>
+      <c r="C43" s="78" t="n"/>
+      <c r="D43" s="77" t="n"/>
+      <c r="E43" s="78" t="n"/>
+      <c r="F43" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="G43" s="74" t="n"/>
+      <c r="H43" s="65">
+        <f>IF(OR(H42="",F45=""),"",IF(H42&gt;F45,2,IF(H42&lt;F45,0,1)))</f>
+        <v/>
+      </c>
+      <c r="I43" s="74" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1" s="19">
+      <c r="A44" s="79" t="n"/>
+      <c r="B44" s="80" t="n"/>
+      <c r="C44" s="81" t="n"/>
+      <c r="D44" s="80" t="n"/>
+      <c r="E44" s="81" t="n"/>
+      <c r="F44" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G44" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="H44" s="65">
+        <f>IF(I42&gt;0,TRUNC(H42/I42,3),"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="65" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1" s="19">
+      <c r="A45" s="70">
+        <f>IF(OR(H12="",F15=""),"",IF(H12&lt;F15,A12,IF(F15&lt;H12,A15,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="B45" s="66" t="n"/>
+      <c r="C45" s="75" t="n"/>
+      <c r="D45" s="66" t="n"/>
+      <c r="E45" s="75" t="n"/>
+      <c r="F45" s="65" t="n"/>
+      <c r="G45" s="65" t="n"/>
+      <c r="H45" s="60" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="I45" s="60" t="inlineStr">
+        <is>
+          <t>Aufn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1" s="19">
+      <c r="A46" s="76" t="n"/>
+      <c r="B46" s="77" t="n"/>
+      <c r="C46" s="78" t="n"/>
+      <c r="D46" s="77" t="n"/>
+      <c r="E46" s="78" t="n"/>
+      <c r="F46" s="65">
+        <f>IF(OR(F45="",H42=""),"",IF(F45&gt;H42,2,IF(F45&lt;H42,0,1)))</f>
+        <v/>
+      </c>
+      <c r="G46" s="74" t="n"/>
+      <c r="H46" s="60" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="I46" s="74" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1" s="19">
+      <c r="A47" s="79" t="n"/>
+      <c r="B47" s="80" t="n"/>
+      <c r="C47" s="81" t="n"/>
+      <c r="D47" s="80" t="n"/>
+      <c r="E47" s="81" t="n"/>
+      <c r="F47" s="65">
+        <f>IF(G45&gt;0,TRUNC(F45/G45,3),"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="65" t="n"/>
+      <c r="H47" s="60" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="I47" s="60" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="77">
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="H24:I26"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F6:G8"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B42:C44"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="H9:I11"/>
+    <mergeCell ref="D45:E47"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="H39:I41"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D15:E17"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="B15:C17"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B27:C29"/>
+    <mergeCell ref="D27:E29"/>
+    <mergeCell ref="F36:G38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="H36:I38"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="D12:E14"/>
+    <mergeCell ref="B30:C32"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="F9:G11"/>
+    <mergeCell ref="B45:C47"/>
+    <mergeCell ref="F39:G41"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="F24:G26"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D42:E44"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D30:E32"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="B12:C14"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="H6:I8"/>
+    <mergeCell ref="F21:G23"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="H21:I23"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B10:C10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add T15 overall ranking worksheet
</commit_message>
<xml_diff>
--- a/nbv_turniermodi_excel/T15_8 Spieler zwei Vierergruppen Kalender-Vorlage.xlsx
+++ b/nbv_turniermodi_excel/T15_8 Spieler zwei Vierergruppen Kalender-Vorlage.xlsx
@@ -10,12 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnehmer" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV Export" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finalrunde" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gesamtrangliste" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau'!$A$1:$P$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Teilnehmer'!$A$1:$F$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'CSV Export'!$A$1:$M$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Finalrunde'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Gesamtrangliste'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -27,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -90,6 +92,18 @@
       <b val="1"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006B2D"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -144,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="46">
+  <borders count="50">
     <border>
       <left/>
       <right/>
@@ -641,12 +655,47 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="center"/>
@@ -845,6 +894,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3750,7 +3826,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="19">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="82" t="inlineStr">
         <is>
           <t>Final- und Platzierungsspiele</t>
         </is>
@@ -3765,7 +3841,7 @@
       <c r="I1" s="71" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1" s="19">
-      <c r="A2" s="68" t="inlineStr">
+      <c r="A2" s="83" t="inlineStr">
         <is>
           <t>Die Spieler werden aus den Gruppenplatzierungen ermittelt. Namen aktualisieren sich nach Eingabe der Gruppenergebnisse.</t>
         </is>
@@ -3780,7 +3856,7 @@
       <c r="I2" s="72" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1" s="19">
-      <c r="A4" s="69" t="inlineStr">
+      <c r="A4" s="84" t="inlineStr">
         <is>
           <t>Halbfinale</t>
         </is>
@@ -4074,7 +4150,7 @@
       </c>
     </row>
     <row r="19" ht="26" customHeight="1" s="19">
-      <c r="A19" s="69" t="inlineStr">
+      <c r="A19" s="84" t="inlineStr">
         <is>
           <t>Platzierung 5-8</t>
         </is>
@@ -4368,7 +4444,7 @@
       </c>
     </row>
     <row r="34" ht="26" customHeight="1" s="19">
-      <c r="A34" s="69" t="inlineStr">
+      <c r="A34" s="84" t="inlineStr">
         <is>
           <t>Endspiele</t>
         </is>
@@ -4743,4 +4819,466 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="19" min="1" max="1"/>
+    <col width="24" customWidth="1" style="19" min="2" max="2"/>
+    <col width="12" customWidth="1" style="19" min="3" max="3"/>
+    <col width="12" customWidth="1" style="19" min="4" max="4"/>
+    <col width="14" customWidth="1" style="19" min="5" max="5"/>
+    <col width="14" customWidth="1" style="19" min="6" max="6"/>
+    <col width="12" customWidth="1" style="19" min="7" max="7"/>
+    <col width="12" customWidth="1" style="19" min="8" max="8"/>
+    <col width="10" customWidth="1" style="19" min="9" max="9"/>
+    <col width="10" customWidth="1" style="19" min="10" max="10"/>
+    <col width="22" customWidth="1" style="19" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="19">
+      <c r="A1" s="85" t="inlineStr">
+        <is>
+          <t>Gesamtrangliste</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="68" t="inlineStr">
+        <is>
+          <t>Platzierung aus Finalrunde; Gruppendaten werden aus dem Tableau übernommen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="86" t="inlineStr">
+        <is>
+          <t>Platz</t>
+        </is>
+      </c>
+      <c r="B3" s="86" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="C3" s="86" t="inlineStr">
+        <is>
+          <t>Pass-Nr.</t>
+        </is>
+      </c>
+      <c r="D3" s="86" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="E3" s="86" t="inlineStr">
+        <is>
+          <t>Gruppenplatz</t>
+        </is>
+      </c>
+      <c r="F3" s="86" t="inlineStr">
+        <is>
+          <t>Partiepunkte</t>
+        </is>
+      </c>
+      <c r="G3" s="86" t="inlineStr">
+        <is>
+          <t>Bälle</t>
+        </is>
+      </c>
+      <c r="H3" s="86" t="inlineStr">
+        <is>
+          <t>Aufnahmen</t>
+        </is>
+      </c>
+      <c r="I3" s="86" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="J3" s="86" t="inlineStr">
+        <is>
+          <t>HS</t>
+        </is>
+      </c>
+      <c r="K3" s="86" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="88">
+        <f>IF(OR(Finalrunde!D36="",Finalrunde!B39=""),"",IF(Finalrunde!D36&gt;Finalrunde!B39,Finalrunde!A36,IF(Finalrunde!B39&gt;Finalrunde!D36,Finalrunde!A39,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B4,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D4" s="90">
+        <f>IF(B4="","",IF(ISNUMBER(MATCH(B4,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B4,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J4" s="89">
+        <f>IF(B4="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B4,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B4,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K4" s="90">
+        <f>IF(B4="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="88">
+        <f>IF(OR(Finalrunde!D36="",Finalrunde!B39=""),"",IF(Finalrunde!D36&lt;Finalrunde!B39,Finalrunde!A36,IF(Finalrunde!B39&lt;Finalrunde!D36,Finalrunde!A39,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B5,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D5" s="90">
+        <f>IF(B5="","",IF(ISNUMBER(MATCH(B5,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B5,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J5" s="89">
+        <f>IF(B5="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B5,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B5,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K5" s="90">
+        <f>IF(B5="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="88">
+        <f>IF(OR(Finalrunde!H42="",Finalrunde!F45=""),"",IF(Finalrunde!H42&gt;Finalrunde!F45,Finalrunde!A42,IF(Finalrunde!F45&gt;Finalrunde!H42,Finalrunde!A45,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B6,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D6" s="90">
+        <f>IF(B6="","",IF(ISNUMBER(MATCH(B6,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B6,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J6" s="89">
+        <f>IF(B6="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B6,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B6,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K6" s="90">
+        <f>IF(B6="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="88">
+        <f>IF(OR(Finalrunde!H42="",Finalrunde!F45=""),"",IF(Finalrunde!H42&lt;Finalrunde!F45,Finalrunde!A42,IF(Finalrunde!F45&lt;Finalrunde!H42,Finalrunde!A45,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B7,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D7" s="90">
+        <f>IF(B7="","",IF(ISNUMBER(MATCH(B7,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B7,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J7" s="89">
+        <f>IF(B7="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B7,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B7,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K7" s="90">
+        <f>IF(B7="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="88">
+        <f>IF(OR(Finalrunde!D21="",Finalrunde!B24=""),"",IF(Finalrunde!D21&gt;Finalrunde!B24,Finalrunde!A21,IF(Finalrunde!B24&gt;Finalrunde!D21,Finalrunde!A24,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B8,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D8" s="90">
+        <f>IF(B8="","",IF(ISNUMBER(MATCH(B8,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B8,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J8" s="89">
+        <f>IF(B8="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B8,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B8,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K8" s="90">
+        <f>IF(B8="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="87" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="88">
+        <f>IF(OR(Finalrunde!D21="",Finalrunde!B24=""),"",IF(Finalrunde!D21&lt;Finalrunde!B24,Finalrunde!A21,IF(Finalrunde!B24&lt;Finalrunde!D21,Finalrunde!A24,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B9,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D9" s="90">
+        <f>IF(B9="","",IF(ISNUMBER(MATCH(B9,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B9,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J9" s="89">
+        <f>IF(B9="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B9,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B9,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K9" s="90">
+        <f>IF(B9="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="87" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="88">
+        <f>IF(OR(Finalrunde!H27="",Finalrunde!F30=""),"",IF(Finalrunde!H27&gt;Finalrunde!F30,Finalrunde!A27,IF(Finalrunde!F30&gt;Finalrunde!H27,Finalrunde!A30,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B10,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D10" s="90">
+        <f>IF(B10="","",IF(ISNUMBER(MATCH(B10,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B10,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J10" s="89">
+        <f>IF(B10="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B10,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B10,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K10" s="90">
+        <f>IF(B10="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="87" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="88">
+        <f>IF(OR(Finalrunde!H27="",Finalrunde!F30=""),"",IF(Finalrunde!H27&lt;Finalrunde!F30,Finalrunde!A27,IF(Finalrunde!F30&lt;Finalrunde!H27,Finalrunde!A30,"Losentscheidung")))</f>
+        <v/>
+      </c>
+      <c r="C11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Teilnehmer!$C$2:$C$9,MATCH(B11,Teilnehmer!$B$2:$B$9,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D11" s="90">
+        <f>IF(B11="","",IF(ISNUMBER(MATCH(B11,Tableau!$A$6:$A$15,0)),"Gruppe 1",IF(ISNUMBER(MATCH(B11,Tableau!$A$22:$A$31,0)),"Gruppe 2","")))</f>
+        <v/>
+      </c>
+      <c r="E11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$O$6:$O$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$O$22:$O$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="F11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$J$6:$J$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$J$22:$J$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="G11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$K$6:$K$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$K$22:$K$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="H11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$L$6:$L$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$L$22:$L$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="I11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$M$6:$M$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$M$22:$M$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="J11" s="89">
+        <f>IF(B11="","",IFERROR(INDEX(Tableau!$N$6:$N$15,MATCH(B11,Tableau!$A$6:$A$15,0)),IFERROR(INDEX(Tableau!$N$22:$N$31,MATCH(B11,Tableau!$A$22:$A$31,0)),"")))</f>
+        <v/>
+      </c>
+      <c r="K11" s="90">
+        <f>IF(B11="Losentscheidung","Bitte manuell klären","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>